<commit_message>
Complete steam and condensate sizing engine with hydraulic validation
</commit_message>
<xml_diff>
--- a/databases/FITTINGS_DB.xlsx
+++ b/databases/FITTINGS_DB.xlsx
@@ -5,16 +5,16 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\SteamBOQ_AI\databases\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Projects_AI\SteamBOQ_AI\databases\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D637D12C-2CB0-458A-A0E4-15463D6DD35B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BB20DA50-E22D-46B5-83A3-B2712DE72471}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="1812" yWindow="1812" windowWidth="17280" windowHeight="8964" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
-    <sheet name="Sheet2" sheetId="2" r:id="rId2"/>
+    <sheet name="Fittings" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="162913"/>
   <extLst>
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="32" uniqueCount="20">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="71" uniqueCount="45">
   <si>
     <t>Component</t>
   </si>
@@ -70,22 +70,97 @@
     <t>Separator</t>
   </si>
   <si>
-    <t>Fitting Type</t>
-  </si>
-  <si>
-    <t>Size</t>
-  </si>
-  <si>
-    <t>Schedule</t>
-  </si>
-  <si>
-    <t>Material</t>
-  </si>
-  <si>
-    <t>Weight</t>
-  </si>
-  <si>
-    <t>Rate</t>
+    <t>Elbow</t>
+  </si>
+  <si>
+    <t>Tee Through</t>
+  </si>
+  <si>
+    <t>Tee</t>
+  </si>
+  <si>
+    <t>Valve</t>
+  </si>
+  <si>
+    <t>Butterfly Valve</t>
+  </si>
+  <si>
+    <t>Y Strainer</t>
+  </si>
+  <si>
+    <t>Strainer</t>
+  </si>
+  <si>
+    <t>Reducer</t>
+  </si>
+  <si>
+    <t>Expansion Joint</t>
+  </si>
+  <si>
+    <t>Expansion</t>
+  </si>
+  <si>
+    <t>Fitting_Code</t>
+  </si>
+  <si>
+    <t>ELBOW_90_LR</t>
+  </si>
+  <si>
+    <t>ELBOW_90_SR</t>
+  </si>
+  <si>
+    <t>TEE_THROUGH</t>
+  </si>
+  <si>
+    <t>TEE_BRANCH</t>
+  </si>
+  <si>
+    <t>EXPANSION_JOINT</t>
+  </si>
+  <si>
+    <t>GATE_VALVE</t>
+  </si>
+  <si>
+    <t>GLOBE_VALVE</t>
+  </si>
+  <si>
+    <t>BALL_VALVE</t>
+  </si>
+  <si>
+    <t>BUTTERFLY_VALVE</t>
+  </si>
+  <si>
+    <t>Y_STRAINER</t>
+  </si>
+  <si>
+    <t>ELBOW_45</t>
+  </si>
+  <si>
+    <t>REDUCER</t>
+  </si>
+  <si>
+    <t>Category</t>
+  </si>
+  <si>
+    <t>90° Long Radius Elbow</t>
+  </si>
+  <si>
+    <t>90° Short Radius Elbow</t>
+  </si>
+  <si>
+    <t>SWING_CHECK</t>
+  </si>
+  <si>
+    <t>Crane TP-410</t>
+  </si>
+  <si>
+    <t>Source</t>
+  </si>
+  <si>
+    <t>Le_over_D</t>
+  </si>
+  <si>
+    <t>Description</t>
   </si>
 </sst>
 </file>
@@ -144,7 +219,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -153,6 +228,12 @@
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -544,90 +625,251 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E31773E1-AABC-4F80-AAD9-CF6802294467}">
-  <dimension ref="A1:F13"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <dimension ref="A1:E14"/>
+  <sheetFormatPr defaultColWidth="21.44140625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="21.5546875" customWidth="1"/>
+    <col min="1" max="1" width="16.6640625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="19.88671875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="9.21875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="9.88671875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A1" t="s">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A1" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="D1" s="4" t="s">
+        <v>43</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A2" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="B2" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="C2" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="B1" t="s">
+      <c r="D2" s="5">
+        <v>30</v>
+      </c>
+      <c r="E2" s="2" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A3" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="B3" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="C3" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="D3" s="5">
+        <v>50</v>
+      </c>
+      <c r="E3" s="2" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A4" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="B4" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="C4" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="D4" s="5">
+        <v>16</v>
+      </c>
+      <c r="E4" s="2" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A5" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="B5" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C5" s="2" t="s">
         <v>16</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D5" s="5">
+        <v>20</v>
+      </c>
+      <c r="E5" s="2" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A6" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="B6" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="C6" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="D6" s="5">
+        <v>60</v>
+      </c>
+      <c r="E6" s="2" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A7" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="B7" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="C7" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="E1" t="s">
+      <c r="D7" s="5">
+        <v>8</v>
+      </c>
+      <c r="E7" s="2" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A8" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="B8" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="C8" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="D8" s="5">
+        <v>340</v>
+      </c>
+      <c r="E8" s="2" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A9" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="B9" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="C9" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="D9" s="5">
+        <v>3</v>
+      </c>
+      <c r="E9" s="2" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="10" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A10" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="B10" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="F1" t="s">
+      <c r="C10" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="D10" s="5">
+        <v>45</v>
+      </c>
+      <c r="E10" s="2" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="11" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A11" s="2" t="s">
+        <v>40</v>
+      </c>
+      <c r="B11" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="C11" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="D11" s="5">
+        <v>100</v>
+      </c>
+      <c r="E11" s="2" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="12" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A12" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="B12" s="2" t="s">
         <v>19</v>
       </c>
-    </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A2" s="2" t="s">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A3" s="2" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A4" s="2" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A5" s="2" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A6" s="2" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A7" s="2" t="s">
+      <c r="C12" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="D12" s="5">
+        <v>100</v>
+      </c>
+      <c r="E12" s="2" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="13" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A13" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="B13" s="2" t="s">
         <v>7</v>
       </c>
-    </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A8" s="2" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A9" s="2" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A10" s="2" t="s">
+      <c r="C13" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="D13" s="5">
+        <v>12</v>
+      </c>
+      <c r="E13" s="2" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="14" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A14" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="B14" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="C14" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="D14" s="5">
         <v>10</v>
       </c>
-    </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A11" s="2" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="12" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A12" s="2" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="13" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A13" s="2" t="s">
-        <v>13</v>
+      <c r="E14" s="2" t="s">
+        <v>41</v>
       </c>
     </row>
   </sheetData>

</xml_diff>